<commit_message>
feat(day1-2): cap nhat build_graph.py dung ban do Q1 OSMnx, dinh vi Hubs va sua load_data
</commit_message>
<xml_diff>
--- a/results/summary_results.xlsx
+++ b/results/summary_results.xlsx
@@ -488,28 +488,28 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3.93</v>
+        <v>3.1</v>
       </c>
       <c r="D2" t="n">
-        <v>587.2</v>
+        <v>271.64</v>
       </c>
       <c r="E2" t="n">
-        <v>1.96</v>
+        <v>1.55</v>
       </c>
       <c r="F2" t="n">
-        <v>1761606.11</v>
+        <v>814907.1899999999</v>
       </c>
       <c r="G2" t="n">
-        <v>5891.66</v>
+        <v>4656.61</v>
       </c>
       <c r="H2" t="n">
-        <v>70.45999999999999</v>
+        <v>32.6</v>
       </c>
       <c r="I2" t="n">
-        <v>0.24</v>
+        <v>0.19</v>
       </c>
       <c r="J2" t="n">
-        <v>299</v>
+        <v>175</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -527,28 +527,28 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3.93</v>
+        <v>3.1</v>
       </c>
       <c r="D3" t="n">
-        <v>587.2</v>
+        <v>271.64</v>
       </c>
       <c r="E3" t="n">
-        <v>1.96</v>
+        <v>1.55</v>
       </c>
       <c r="F3" t="n">
-        <v>1761606.11</v>
+        <v>814907.1899999999</v>
       </c>
       <c r="G3" t="n">
-        <v>5891.66</v>
+        <v>4656.61</v>
       </c>
       <c r="H3" t="n">
-        <v>70.45999999999999</v>
+        <v>32.6</v>
       </c>
       <c r="I3" t="n">
-        <v>0.24</v>
+        <v>0.19</v>
       </c>
       <c r="J3" t="n">
-        <v>299</v>
+        <v>175</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -566,28 +566,28 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3.93</v>
+        <v>3.1</v>
       </c>
       <c r="D4" t="n">
-        <v>587.2</v>
+        <v>271.64</v>
       </c>
       <c r="E4" t="n">
-        <v>1.96</v>
+        <v>1.55</v>
       </c>
       <c r="F4" t="n">
-        <v>1761606.11</v>
+        <v>814907.1899999999</v>
       </c>
       <c r="G4" t="n">
-        <v>5891.66</v>
+        <v>4656.61</v>
       </c>
       <c r="H4" t="n">
-        <v>70.45999999999999</v>
+        <v>32.6</v>
       </c>
       <c r="I4" t="n">
-        <v>0.24</v>
+        <v>0.19</v>
       </c>
       <c r="J4" t="n">
-        <v>299</v>
+        <v>175</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -605,28 +605,28 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3.93</v>
+        <v>3.1</v>
       </c>
       <c r="D5" t="n">
-        <v>587.2</v>
+        <v>271.64</v>
       </c>
       <c r="E5" t="n">
-        <v>1.96</v>
+        <v>1.55</v>
       </c>
       <c r="F5" t="n">
-        <v>1761606.11</v>
+        <v>814907.1899999999</v>
       </c>
       <c r="G5" t="n">
-        <v>5891.66</v>
+        <v>4656.61</v>
       </c>
       <c r="H5" t="n">
-        <v>70.45999999999999</v>
+        <v>32.6</v>
       </c>
       <c r="I5" t="n">
-        <v>0.24</v>
+        <v>0.19</v>
       </c>
       <c r="J5" t="n">
-        <v>299</v>
+        <v>175</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -644,28 +644,28 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>9.82</v>
+        <v>7.76</v>
       </c>
       <c r="D6" t="n">
-        <v>587.2</v>
+        <v>271.64</v>
       </c>
       <c r="E6" t="n">
-        <v>1.96</v>
+        <v>1.55</v>
       </c>
       <c r="F6" t="n">
-        <v>1761606.11</v>
+        <v>814907.1899999999</v>
       </c>
       <c r="G6" t="n">
-        <v>5891.66</v>
+        <v>4656.61</v>
       </c>
       <c r="H6" t="n">
-        <v>70.45999999999999</v>
+        <v>32.6</v>
       </c>
       <c r="I6" t="n">
-        <v>0.24</v>
+        <v>0.19</v>
       </c>
       <c r="J6" t="n">
-        <v>299</v>
+        <v>175</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
@@ -683,28 +683,28 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>9.82</v>
+        <v>7.76</v>
       </c>
       <c r="D7" t="n">
-        <v>587.2</v>
+        <v>271.64</v>
       </c>
       <c r="E7" t="n">
-        <v>1.96</v>
+        <v>1.55</v>
       </c>
       <c r="F7" t="n">
-        <v>1761606.11</v>
+        <v>814907.1899999999</v>
       </c>
       <c r="G7" t="n">
-        <v>5891.66</v>
+        <v>4656.61</v>
       </c>
       <c r="H7" t="n">
-        <v>70.45999999999999</v>
+        <v>32.6</v>
       </c>
       <c r="I7" t="n">
-        <v>0.24</v>
+        <v>0.19</v>
       </c>
       <c r="J7" t="n">
-        <v>299</v>
+        <v>175</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -722,28 +722,28 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>9.82</v>
+        <v>7.76</v>
       </c>
       <c r="D8" t="n">
-        <v>587.2</v>
+        <v>271.64</v>
       </c>
       <c r="E8" t="n">
-        <v>1.96</v>
+        <v>1.55</v>
       </c>
       <c r="F8" t="n">
-        <v>1761606.11</v>
+        <v>814907.1899999999</v>
       </c>
       <c r="G8" t="n">
-        <v>5891.66</v>
+        <v>4656.61</v>
       </c>
       <c r="H8" t="n">
-        <v>70.45999999999999</v>
+        <v>32.6</v>
       </c>
       <c r="I8" t="n">
-        <v>0.24</v>
+        <v>0.19</v>
       </c>
       <c r="J8" t="n">
-        <v>299</v>
+        <v>175</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -761,28 +761,28 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>9.82</v>
+        <v>7.76</v>
       </c>
       <c r="D9" t="n">
-        <v>587.2</v>
+        <v>271.64</v>
       </c>
       <c r="E9" t="n">
-        <v>1.96</v>
+        <v>1.55</v>
       </c>
       <c r="F9" t="n">
-        <v>1761606.11</v>
+        <v>814907.1899999999</v>
       </c>
       <c r="G9" t="n">
-        <v>5891.66</v>
+        <v>4656.61</v>
       </c>
       <c r="H9" t="n">
-        <v>70.45999999999999</v>
+        <v>32.6</v>
       </c>
       <c r="I9" t="n">
-        <v>0.24</v>
+        <v>0.19</v>
       </c>
       <c r="J9" t="n">
-        <v>299</v>
+        <v>175</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -871,13 +871,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3.93</v>
+        <v>3.1</v>
       </c>
       <c r="E2" t="n">
-        <v>70.45999999999999</v>
+        <v>32.6</v>
       </c>
       <c r="F2" t="n">
-        <v>5891.66</v>
+        <v>4656.61</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -909,13 +909,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3.93</v>
+        <v>3.1</v>
       </c>
       <c r="E3" t="n">
-        <v>70.45999999999999</v>
+        <v>32.6</v>
       </c>
       <c r="F3" t="n">
-        <v>5891.66</v>
+        <v>4656.61</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -947,13 +947,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3.93</v>
+        <v>3.1</v>
       </c>
       <c r="E4" t="n">
-        <v>70.45999999999999</v>
+        <v>32.6</v>
       </c>
       <c r="F4" t="n">
-        <v>5891.66</v>
+        <v>4656.61</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -985,13 +985,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>3.93</v>
+        <v>3.1</v>
       </c>
       <c r="E5" t="n">
-        <v>70.45999999999999</v>
+        <v>32.6</v>
       </c>
       <c r="F5" t="n">
-        <v>5891.66</v>
+        <v>4656.61</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -1023,13 +1023,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>9.82</v>
+        <v>7.76</v>
       </c>
       <c r="E6" t="n">
-        <v>70.45999999999999</v>
+        <v>32.6</v>
       </c>
       <c r="F6" t="n">
-        <v>5891.66</v>
+        <v>4656.61</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -1061,13 +1061,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>9.82</v>
+        <v>7.76</v>
       </c>
       <c r="E7" t="n">
-        <v>70.45999999999999</v>
+        <v>32.6</v>
       </c>
       <c r="F7" t="n">
-        <v>5891.66</v>
+        <v>4656.61</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -1099,13 +1099,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>9.82</v>
+        <v>7.76</v>
       </c>
       <c r="E8" t="n">
-        <v>70.45999999999999</v>
+        <v>32.6</v>
       </c>
       <c r="F8" t="n">
-        <v>5891.66</v>
+        <v>4656.61</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -1137,13 +1137,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>9.82</v>
+        <v>7.76</v>
       </c>
       <c r="E9" t="n">
-        <v>70.45999999999999</v>
+        <v>32.6</v>
       </c>
       <c r="F9" t="n">
-        <v>5891.66</v>
+        <v>4656.61</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -1241,31 +1241,31 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>11.72</v>
+        <v>4.99</v>
       </c>
       <c r="D2" t="n">
-        <v>1832.42</v>
+        <v>728.72</v>
       </c>
       <c r="E2" t="n">
-        <v>6.11</v>
+        <v>2.5</v>
       </c>
       <c r="F2" t="n">
-        <v>4161933.71</v>
+        <v>2186154.16</v>
       </c>
       <c r="G2" t="n">
-        <v>13873.11</v>
+        <v>7486.83</v>
       </c>
       <c r="H2" t="n">
-        <v>127.65</v>
+        <v>87.44</v>
       </c>
       <c r="I2" t="n">
-        <v>0.43</v>
+        <v>0.3</v>
       </c>
       <c r="J2" t="n">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="K2" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1280,31 +1280,31 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>11.72</v>
+        <v>4.99</v>
       </c>
       <c r="D3" t="n">
-        <v>1832.42</v>
+        <v>728.72</v>
       </c>
       <c r="E3" t="n">
-        <v>6.11</v>
+        <v>2.5</v>
       </c>
       <c r="F3" t="n">
-        <v>4161933.71</v>
+        <v>2186154.16</v>
       </c>
       <c r="G3" t="n">
-        <v>13873.11</v>
+        <v>7486.83</v>
       </c>
       <c r="H3" t="n">
-        <v>127.65</v>
+        <v>87.44</v>
       </c>
       <c r="I3" t="n">
-        <v>0.43</v>
+        <v>0.3</v>
       </c>
       <c r="J3" t="n">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="K3" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -1319,28 +1319,28 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>12.65</v>
+        <v>4.99</v>
       </c>
       <c r="D4" t="n">
-        <v>1897.84</v>
+        <v>728.72</v>
       </c>
       <c r="E4" t="n">
-        <v>6.33</v>
+        <v>2.5</v>
       </c>
       <c r="F4" t="n">
-        <v>5693519.39</v>
+        <v>2186154.16</v>
       </c>
       <c r="G4" t="n">
-        <v>18978.4</v>
+        <v>7486.83</v>
       </c>
       <c r="H4" t="n">
-        <v>227.74</v>
+        <v>87.44</v>
       </c>
       <c r="I4" t="n">
-        <v>0.76</v>
+        <v>0.3</v>
       </c>
       <c r="J4" t="n">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -1358,28 +1358,28 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>12.65</v>
+        <v>4.99</v>
       </c>
       <c r="D5" t="n">
-        <v>1897.84</v>
+        <v>728.72</v>
       </c>
       <c r="E5" t="n">
-        <v>6.33</v>
+        <v>2.5</v>
       </c>
       <c r="F5" t="n">
-        <v>5693519.39</v>
+        <v>2186154.16</v>
       </c>
       <c r="G5" t="n">
-        <v>18978.4</v>
+        <v>7486.83</v>
       </c>
       <c r="H5" t="n">
-        <v>227.74</v>
+        <v>87.44</v>
       </c>
       <c r="I5" t="n">
-        <v>0.76</v>
+        <v>0.3</v>
       </c>
       <c r="J5" t="n">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -1397,31 +1397,31 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>18.16</v>
+        <v>11.3</v>
       </c>
       <c r="D6" t="n">
-        <v>1986.65</v>
+        <v>737.11</v>
       </c>
       <c r="E6" t="n">
-        <v>6.62</v>
+        <v>2.52</v>
       </c>
       <c r="F6" t="n">
-        <v>4240068.04</v>
+        <v>3352809.12</v>
       </c>
       <c r="G6" t="n">
-        <v>14133.56</v>
+        <v>11482.22</v>
       </c>
       <c r="H6" t="n">
-        <v>93.65000000000001</v>
+        <v>64.65000000000001</v>
       </c>
       <c r="I6" t="n">
-        <v>0.31</v>
+        <v>0.22</v>
       </c>
       <c r="J6" t="n">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="K6" t="n">
-        <v>174</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7">
@@ -1436,31 +1436,31 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>18.16</v>
+        <v>11.3</v>
       </c>
       <c r="D7" t="n">
-        <v>1986.65</v>
+        <v>737.11</v>
       </c>
       <c r="E7" t="n">
-        <v>6.62</v>
+        <v>2.52</v>
       </c>
       <c r="F7" t="n">
-        <v>4240068.04</v>
+        <v>3352809.12</v>
       </c>
       <c r="G7" t="n">
-        <v>14133.56</v>
+        <v>11482.22</v>
       </c>
       <c r="H7" t="n">
-        <v>93.65000000000001</v>
+        <v>64.65000000000001</v>
       </c>
       <c r="I7" t="n">
-        <v>0.31</v>
+        <v>0.22</v>
       </c>
       <c r="J7" t="n">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="K7" t="n">
-        <v>174</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8">
@@ -1475,31 +1475,31 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>29.17</v>
+        <v>12.48</v>
       </c>
       <c r="D8" t="n">
-        <v>1949.45</v>
+        <v>728.72</v>
       </c>
       <c r="E8" t="n">
-        <v>6.5</v>
+        <v>2.5</v>
       </c>
       <c r="F8" t="n">
-        <v>5057029.9</v>
+        <v>2186154.16</v>
       </c>
       <c r="G8" t="n">
-        <v>16856.77</v>
+        <v>7486.83</v>
       </c>
       <c r="H8" t="n">
-        <v>181.27</v>
+        <v>87.44</v>
       </c>
       <c r="I8" t="n">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
       <c r="J8" t="n">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="K8" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1514,28 +1514,28 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>31.63</v>
+        <v>12.48</v>
       </c>
       <c r="D9" t="n">
-        <v>1897.84</v>
+        <v>728.72</v>
       </c>
       <c r="E9" t="n">
-        <v>6.33</v>
+        <v>2.5</v>
       </c>
       <c r="F9" t="n">
-        <v>5693519.39</v>
+        <v>2186154.16</v>
       </c>
       <c r="G9" t="n">
-        <v>18978.4</v>
+        <v>7486.83</v>
       </c>
       <c r="H9" t="n">
-        <v>227.74</v>
+        <v>87.44</v>
       </c>
       <c r="I9" t="n">
-        <v>0.76</v>
+        <v>0.3</v>
       </c>
       <c r="J9" t="n">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -1624,25 +1624,25 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>11.72</v>
+        <v>4.99</v>
       </c>
       <c r="E2" t="n">
-        <v>127.65</v>
+        <v>87.44</v>
       </c>
       <c r="F2" t="n">
-        <v>13873.11</v>
+        <v>7486.83</v>
       </c>
       <c r="G2" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>7.4</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>43.9</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>26.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1662,25 +1662,25 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>11.72</v>
+        <v>4.99</v>
       </c>
       <c r="E3" t="n">
-        <v>127.65</v>
+        <v>87.44</v>
       </c>
       <c r="F3" t="n">
-        <v>13873.11</v>
+        <v>7486.83</v>
       </c>
       <c r="G3" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>7.4</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>43.9</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>26.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>12.65</v>
+        <v>4.99</v>
       </c>
       <c r="E4" t="n">
-        <v>227.74</v>
+        <v>87.44</v>
       </c>
       <c r="F4" t="n">
-        <v>18978.4</v>
+        <v>7486.83</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -1738,13 +1738,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>12.65</v>
+        <v>4.99</v>
       </c>
       <c r="E5" t="n">
-        <v>227.74</v>
+        <v>87.44</v>
       </c>
       <c r="F5" t="n">
-        <v>18978.4</v>
+        <v>7486.83</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -1776,25 +1776,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>18.16</v>
+        <v>11.3</v>
       </c>
       <c r="E6" t="n">
-        <v>93.65000000000001</v>
+        <v>64.65000000000001</v>
       </c>
       <c r="F6" t="n">
-        <v>14133.56</v>
+        <v>11482.22</v>
       </c>
       <c r="G6" t="n">
-        <v>174</v>
+        <v>123</v>
       </c>
       <c r="H6" t="n">
-        <v>42.6</v>
+        <v>9.5</v>
       </c>
       <c r="I6" t="n">
-        <v>58.9</v>
+        <v>26.1</v>
       </c>
       <c r="J6" t="n">
-        <v>25.5</v>
+        <v>-53.4</v>
       </c>
     </row>
     <row r="7">
@@ -1814,25 +1814,25 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>18.16</v>
+        <v>11.3</v>
       </c>
       <c r="E7" t="n">
-        <v>93.65000000000001</v>
+        <v>64.65000000000001</v>
       </c>
       <c r="F7" t="n">
-        <v>14133.56</v>
+        <v>11482.22</v>
       </c>
       <c r="G7" t="n">
-        <v>174</v>
+        <v>123</v>
       </c>
       <c r="H7" t="n">
-        <v>42.6</v>
+        <v>9.5</v>
       </c>
       <c r="I7" t="n">
-        <v>58.9</v>
+        <v>26.1</v>
       </c>
       <c r="J7" t="n">
-        <v>25.5</v>
+        <v>-53.4</v>
       </c>
     </row>
     <row r="8">
@@ -1852,25 +1852,25 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>29.17</v>
+        <v>12.48</v>
       </c>
       <c r="E8" t="n">
-        <v>181.27</v>
+        <v>87.44</v>
       </c>
       <c r="F8" t="n">
-        <v>16856.77</v>
+        <v>7486.83</v>
       </c>
       <c r="G8" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>7.8</v>
+        <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>20.4</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>11.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1890,13 +1890,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>31.63</v>
+        <v>12.48</v>
       </c>
       <c r="E9" t="n">
-        <v>227.74</v>
+        <v>87.44</v>
       </c>
       <c r="F9" t="n">
-        <v>18978.4</v>
+        <v>7486.83</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
fix: fix missing dependencies, dynamic path resolution, and integrate simulation step
</commit_message>
<xml_diff>
--- a/results/summary_results.xlsx
+++ b/results/summary_results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI_nearest" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improve_nearest" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI_centralized" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Improve_centralized" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="KPI_nearest" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Improve_nearest" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="KPI_centralized" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Improve_centralized" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -488,28 +488,28 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3.44</v>
+        <v>5.66</v>
       </c>
       <c r="D2" t="n">
-        <v>301.31</v>
+        <v>497.89</v>
       </c>
       <c r="E2" t="n">
-        <v>1.72</v>
+        <v>2.83</v>
       </c>
       <c r="F2" t="n">
-        <v>903920.67</v>
+        <v>1493661.37</v>
       </c>
       <c r="G2" t="n">
-        <v>5165.26</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>36.16</v>
+        <v>59.75</v>
       </c>
       <c r="I2" t="n">
-        <v>0.21</v>
+        <v>0.34</v>
       </c>
       <c r="J2" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -527,28 +527,28 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3.44</v>
+        <v>5.66</v>
       </c>
       <c r="D3" t="n">
-        <v>301.31</v>
+        <v>497.89</v>
       </c>
       <c r="E3" t="n">
-        <v>1.72</v>
+        <v>2.83</v>
       </c>
       <c r="F3" t="n">
-        <v>903920.67</v>
+        <v>1493661.37</v>
       </c>
       <c r="G3" t="n">
-        <v>5165.26</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>36.16</v>
+        <v>59.75</v>
       </c>
       <c r="I3" t="n">
-        <v>0.21</v>
+        <v>0.34</v>
       </c>
       <c r="J3" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -566,28 +566,28 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3.44</v>
+        <v>5.66</v>
       </c>
       <c r="D4" t="n">
-        <v>301.31</v>
+        <v>497.89</v>
       </c>
       <c r="E4" t="n">
-        <v>1.72</v>
+        <v>2.83</v>
       </c>
       <c r="F4" t="n">
-        <v>903920.67</v>
+        <v>1493661.37</v>
       </c>
       <c r="G4" t="n">
-        <v>5165.26</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>36.16</v>
+        <v>59.75</v>
       </c>
       <c r="I4" t="n">
-        <v>0.21</v>
+        <v>0.34</v>
       </c>
       <c r="J4" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -605,28 +605,28 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>3.44</v>
+        <v>5.66</v>
       </c>
       <c r="D5" t="n">
-        <v>301.31</v>
+        <v>497.89</v>
       </c>
       <c r="E5" t="n">
-        <v>1.72</v>
+        <v>2.83</v>
       </c>
       <c r="F5" t="n">
-        <v>903920.67</v>
+        <v>1493661.37</v>
       </c>
       <c r="G5" t="n">
-        <v>5165.26</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>36.16</v>
+        <v>59.75</v>
       </c>
       <c r="I5" t="n">
-        <v>0.21</v>
+        <v>0.34</v>
       </c>
       <c r="J5" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -644,31 +644,31 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>8.609999999999999</v>
+        <v>14.03</v>
       </c>
       <c r="D6" t="n">
-        <v>301.31</v>
+        <v>502.09</v>
       </c>
       <c r="E6" t="n">
-        <v>1.72</v>
+        <v>2.85</v>
       </c>
       <c r="F6" t="n">
-        <v>903920.67</v>
+        <v>1626918.7</v>
       </c>
       <c r="G6" t="n">
-        <v>5165.26</v>
+        <v>9243.860000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>36.16</v>
+        <v>57.74</v>
       </c>
       <c r="I6" t="n">
-        <v>0.21</v>
+        <v>0.33</v>
       </c>
       <c r="J6" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -683,31 +683,31 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>8.609999999999999</v>
+        <v>14.03</v>
       </c>
       <c r="D7" t="n">
-        <v>301.31</v>
+        <v>502.09</v>
       </c>
       <c r="E7" t="n">
-        <v>1.72</v>
+        <v>2.85</v>
       </c>
       <c r="F7" t="n">
-        <v>903920.67</v>
+        <v>1626918.7</v>
       </c>
       <c r="G7" t="n">
-        <v>5165.26</v>
+        <v>9243.860000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>36.16</v>
+        <v>57.74</v>
       </c>
       <c r="I7" t="n">
-        <v>0.21</v>
+        <v>0.33</v>
       </c>
       <c r="J7" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
@@ -722,28 +722,28 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>8.609999999999999</v>
+        <v>14.14</v>
       </c>
       <c r="D8" t="n">
-        <v>301.31</v>
+        <v>497.89</v>
       </c>
       <c r="E8" t="n">
-        <v>1.72</v>
+        <v>2.83</v>
       </c>
       <c r="F8" t="n">
-        <v>903920.67</v>
+        <v>1493661.37</v>
       </c>
       <c r="G8" t="n">
-        <v>5165.26</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>36.16</v>
+        <v>59.75</v>
       </c>
       <c r="I8" t="n">
-        <v>0.21</v>
+        <v>0.34</v>
       </c>
       <c r="J8" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -761,28 +761,28 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>8.609999999999999</v>
+        <v>14.14</v>
       </c>
       <c r="D9" t="n">
-        <v>301.31</v>
+        <v>497.89</v>
       </c>
       <c r="E9" t="n">
-        <v>1.72</v>
+        <v>2.83</v>
       </c>
       <c r="F9" t="n">
-        <v>903920.67</v>
+        <v>1493661.37</v>
       </c>
       <c r="G9" t="n">
-        <v>5165.26</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>36.16</v>
+        <v>59.75</v>
       </c>
       <c r="I9" t="n">
-        <v>0.21</v>
+        <v>0.34</v>
       </c>
       <c r="J9" t="n">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -871,13 +871,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3.44</v>
+        <v>5.66</v>
       </c>
       <c r="E2" t="n">
-        <v>36.16</v>
+        <v>59.75</v>
       </c>
       <c r="F2" t="n">
-        <v>5165.26</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -909,13 +909,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3.44</v>
+        <v>5.66</v>
       </c>
       <c r="E3" t="n">
-        <v>36.16</v>
+        <v>59.75</v>
       </c>
       <c r="F3" t="n">
-        <v>5165.26</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -947,13 +947,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3.44</v>
+        <v>5.66</v>
       </c>
       <c r="E4" t="n">
-        <v>36.16</v>
+        <v>59.75</v>
       </c>
       <c r="F4" t="n">
-        <v>5165.26</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -985,13 +985,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>3.44</v>
+        <v>5.66</v>
       </c>
       <c r="E5" t="n">
-        <v>36.16</v>
+        <v>59.75</v>
       </c>
       <c r="F5" t="n">
-        <v>5165.26</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -1023,25 +1023,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>8.609999999999999</v>
+        <v>14.03</v>
       </c>
       <c r="E6" t="n">
-        <v>36.16</v>
+        <v>57.74</v>
       </c>
       <c r="F6" t="n">
-        <v>5165.26</v>
+        <v>9243.860000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>-8.9</v>
       </c>
     </row>
     <row r="7">
@@ -1061,25 +1061,25 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>8.609999999999999</v>
+        <v>14.03</v>
       </c>
       <c r="E7" t="n">
-        <v>36.16</v>
+        <v>57.74</v>
       </c>
       <c r="F7" t="n">
-        <v>5165.26</v>
+        <v>9243.860000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>-8.9</v>
       </c>
     </row>
     <row r="8">
@@ -1099,13 +1099,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>8.609999999999999</v>
+        <v>14.14</v>
       </c>
       <c r="E8" t="n">
-        <v>36.16</v>
+        <v>59.75</v>
       </c>
       <c r="F8" t="n">
-        <v>5165.26</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -1137,13 +1137,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>8.609999999999999</v>
+        <v>14.14</v>
       </c>
       <c r="E9" t="n">
-        <v>36.16</v>
+        <v>59.75</v>
       </c>
       <c r="F9" t="n">
-        <v>5165.26</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -1241,28 +1241,28 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4.01</v>
+        <v>5.66</v>
       </c>
       <c r="D2" t="n">
-        <v>583.75</v>
+        <v>497.89</v>
       </c>
       <c r="E2" t="n">
-        <v>2.01</v>
+        <v>2.83</v>
       </c>
       <c r="F2" t="n">
-        <v>1751264.21</v>
+        <v>1493661.37</v>
       </c>
       <c r="G2" t="n">
-        <v>6018.09</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>70.05</v>
+        <v>59.75</v>
       </c>
       <c r="I2" t="n">
-        <v>0.24</v>
+        <v>0.34</v>
       </c>
       <c r="J2" t="n">
-        <v>291</v>
+        <v>176</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -1280,28 +1280,28 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4.01</v>
+        <v>5.66</v>
       </c>
       <c r="D3" t="n">
-        <v>583.75</v>
+        <v>497.89</v>
       </c>
       <c r="E3" t="n">
-        <v>2.01</v>
+        <v>2.83</v>
       </c>
       <c r="F3" t="n">
-        <v>1751264.21</v>
+        <v>1493661.37</v>
       </c>
       <c r="G3" t="n">
-        <v>6018.09</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>70.05</v>
+        <v>59.75</v>
       </c>
       <c r="I3" t="n">
-        <v>0.24</v>
+        <v>0.34</v>
       </c>
       <c r="J3" t="n">
-        <v>291</v>
+        <v>176</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -1319,28 +1319,28 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>4.01</v>
+        <v>5.66</v>
       </c>
       <c r="D4" t="n">
-        <v>583.75</v>
+        <v>497.89</v>
       </c>
       <c r="E4" t="n">
-        <v>2.01</v>
+        <v>2.83</v>
       </c>
       <c r="F4" t="n">
-        <v>1751264.21</v>
+        <v>1493661.37</v>
       </c>
       <c r="G4" t="n">
-        <v>6018.09</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>70.05</v>
+        <v>59.75</v>
       </c>
       <c r="I4" t="n">
-        <v>0.24</v>
+        <v>0.34</v>
       </c>
       <c r="J4" t="n">
-        <v>291</v>
+        <v>176</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -1358,28 +1358,28 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4.01</v>
+        <v>5.66</v>
       </c>
       <c r="D5" t="n">
-        <v>583.75</v>
+        <v>497.89</v>
       </c>
       <c r="E5" t="n">
-        <v>2.01</v>
+        <v>2.83</v>
       </c>
       <c r="F5" t="n">
-        <v>1751264.21</v>
+        <v>1493661.37</v>
       </c>
       <c r="G5" t="n">
-        <v>6018.09</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>70.05</v>
+        <v>59.75</v>
       </c>
       <c r="I5" t="n">
-        <v>0.24</v>
+        <v>0.34</v>
       </c>
       <c r="J5" t="n">
-        <v>291</v>
+        <v>176</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -1397,31 +1397,31 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10.03</v>
+        <v>14.03</v>
       </c>
       <c r="D6" t="n">
-        <v>583.75</v>
+        <v>502.09</v>
       </c>
       <c r="E6" t="n">
-        <v>2.01</v>
+        <v>2.85</v>
       </c>
       <c r="F6" t="n">
-        <v>1751264.21</v>
+        <v>1626918.7</v>
       </c>
       <c r="G6" t="n">
-        <v>6018.09</v>
+        <v>9243.860000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>70.05</v>
+        <v>57.74</v>
       </c>
       <c r="I6" t="n">
-        <v>0.24</v>
+        <v>0.33</v>
       </c>
       <c r="J6" t="n">
-        <v>291</v>
+        <v>176</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -1436,31 +1436,31 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>10.03</v>
+        <v>14.03</v>
       </c>
       <c r="D7" t="n">
-        <v>583.75</v>
+        <v>502.09</v>
       </c>
       <c r="E7" t="n">
-        <v>2.01</v>
+        <v>2.85</v>
       </c>
       <c r="F7" t="n">
-        <v>1751264.21</v>
+        <v>1626918.7</v>
       </c>
       <c r="G7" t="n">
-        <v>6018.09</v>
+        <v>9243.860000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>70.05</v>
+        <v>57.74</v>
       </c>
       <c r="I7" t="n">
-        <v>0.24</v>
+        <v>0.33</v>
       </c>
       <c r="J7" t="n">
-        <v>291</v>
+        <v>176</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
@@ -1475,28 +1475,28 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>10.03</v>
+        <v>14.14</v>
       </c>
       <c r="D8" t="n">
-        <v>583.75</v>
+        <v>497.89</v>
       </c>
       <c r="E8" t="n">
-        <v>2.01</v>
+        <v>2.83</v>
       </c>
       <c r="F8" t="n">
-        <v>1751264.21</v>
+        <v>1493661.37</v>
       </c>
       <c r="G8" t="n">
-        <v>6018.09</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>70.05</v>
+        <v>59.75</v>
       </c>
       <c r="I8" t="n">
-        <v>0.24</v>
+        <v>0.34</v>
       </c>
       <c r="J8" t="n">
-        <v>291</v>
+        <v>176</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -1514,28 +1514,28 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>10.03</v>
+        <v>14.14</v>
       </c>
       <c r="D9" t="n">
-        <v>583.75</v>
+        <v>497.89</v>
       </c>
       <c r="E9" t="n">
-        <v>2.01</v>
+        <v>2.83</v>
       </c>
       <c r="F9" t="n">
-        <v>1751264.21</v>
+        <v>1493661.37</v>
       </c>
       <c r="G9" t="n">
-        <v>6018.09</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>70.05</v>
+        <v>59.75</v>
       </c>
       <c r="I9" t="n">
-        <v>0.24</v>
+        <v>0.34</v>
       </c>
       <c r="J9" t="n">
-        <v>291</v>
+        <v>176</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -1624,13 +1624,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4.01</v>
+        <v>5.66</v>
       </c>
       <c r="E2" t="n">
-        <v>70.05</v>
+        <v>59.75</v>
       </c>
       <c r="F2" t="n">
-        <v>6018.09</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -1662,13 +1662,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>4.01</v>
+        <v>5.66</v>
       </c>
       <c r="E3" t="n">
-        <v>70.05</v>
+        <v>59.75</v>
       </c>
       <c r="F3" t="n">
-        <v>6018.09</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -1700,13 +1700,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>4.01</v>
+        <v>5.66</v>
       </c>
       <c r="E4" t="n">
-        <v>70.05</v>
+        <v>59.75</v>
       </c>
       <c r="F4" t="n">
-        <v>6018.09</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -1738,13 +1738,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>4.01</v>
+        <v>5.66</v>
       </c>
       <c r="E5" t="n">
-        <v>70.05</v>
+        <v>59.75</v>
       </c>
       <c r="F5" t="n">
-        <v>6018.09</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -1776,25 +1776,25 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>10.03</v>
+        <v>14.03</v>
       </c>
       <c r="E6" t="n">
-        <v>70.05</v>
+        <v>57.74</v>
       </c>
       <c r="F6" t="n">
-        <v>6018.09</v>
+        <v>9243.860000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>-8.9</v>
       </c>
     </row>
     <row r="7">
@@ -1814,25 +1814,25 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>10.03</v>
+        <v>14.03</v>
       </c>
       <c r="E7" t="n">
-        <v>70.05</v>
+        <v>57.74</v>
       </c>
       <c r="F7" t="n">
-        <v>6018.09</v>
+        <v>9243.860000000001</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>-8.9</v>
       </c>
     </row>
     <row r="8">
@@ -1852,13 +1852,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>10.03</v>
+        <v>14.14</v>
       </c>
       <c r="E8" t="n">
-        <v>70.05</v>
+        <v>59.75</v>
       </c>
       <c r="F8" t="n">
-        <v>6018.09</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -1890,13 +1890,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>10.03</v>
+        <v>14.14</v>
       </c>
       <c r="E9" t="n">
-        <v>70.05</v>
+        <v>59.75</v>
       </c>
       <c r="F9" t="n">
-        <v>6018.09</v>
+        <v>8486.709999999999</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>

</xml_diff>